<commit_message>
fix: Move legal basis form position in bulk upload
</commit_message>
<xml_diff>
--- a/src/test/resource/Bulk_Upload_Awards_Template_local_errors.xlsx
+++ b/src/test/resource/Bulk_Upload_Awards_Template_local_errors.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\BEIS\source\transparency-db-publishing-subsidies-service\src\test\resource\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1381028-AFC2-4A79-8CE8-CF46B6B01DA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CF521C0-8C88-43FB-A6F1-4CFB4AA1048B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1312,6 +1312,9 @@
     <xf numFmtId="49" fontId="13" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1329,9 +1332,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1688,14 +1688,14 @@
       <c r="H1" s="19" t="s">
         <v>165</v>
       </c>
-      <c r="I1" s="34" t="s">
+      <c r="I1" s="38" t="s">
+        <v>208</v>
+      </c>
+      <c r="J1" s="34" t="s">
         <v>193</v>
       </c>
-      <c r="J1" s="35" t="s">
+      <c r="K1" s="35" t="s">
         <v>194</v>
-      </c>
-      <c r="K1" s="38" t="s">
-        <v>208</v>
       </c>
       <c r="L1" s="38" t="s">
         <v>207</v>
@@ -1762,13 +1762,13 @@
       <c r="G2" s="24"/>
       <c r="H2" s="24"/>
       <c r="I2" s="24" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="J2" s="24" t="s">
         <v>195</v>
       </c>
       <c r="K2" s="24" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="L2" s="24"/>
       <c r="M2" s="22" t="s">
@@ -1833,13 +1833,13 @@
       <c r="G3" s="24"/>
       <c r="H3" s="24"/>
       <c r="I3" s="24" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="J3" s="24" t="s">
         <v>195</v>
       </c>
       <c r="K3" s="24" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="L3" s="24" t="s">
         <v>168</v>
@@ -1897,7 +1897,7 @@
       <c r="D4" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="E4" s="45" t="s">
+      <c r="E4" s="39" t="s">
         <v>211</v>
       </c>
       <c r="F4" s="24" t="s">
@@ -1906,13 +1906,13 @@
       <c r="G4" s="24"/>
       <c r="H4" s="24"/>
       <c r="I4" s="24" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="J4" s="24" t="s">
         <v>195</v>
       </c>
       <c r="K4" s="24" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="L4" s="24" t="s">
         <v>167</v>
@@ -1972,18 +1972,18 @@
       <c r="D5" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="E5" s="45"/>
+      <c r="E5" s="39"/>
       <c r="F5" s="24"/>
       <c r="G5" s="24"/>
       <c r="H5" s="24"/>
       <c r="I5" s="24" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="J5" s="24" t="s">
         <v>195</v>
       </c>
       <c r="K5" s="24" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="L5" s="24" t="s">
         <v>168</v>
@@ -2041,7 +2041,7 @@
       <c r="D6" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="E6" s="45" t="s">
+      <c r="E6" s="39" t="s">
         <v>211</v>
       </c>
       <c r="F6" s="24"/>
@@ -2050,13 +2050,13 @@
       </c>
       <c r="H6" s="24"/>
       <c r="I6" s="24" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="J6" s="24" t="s">
         <v>195</v>
       </c>
       <c r="K6" s="24" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="L6" s="24" t="s">
         <v>167</v>
@@ -2116,18 +2116,18 @@
       <c r="D7" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="E7" s="45"/>
+      <c r="E7" s="39"/>
       <c r="F7" s="24"/>
       <c r="G7" s="24"/>
       <c r="H7" s="24"/>
       <c r="I7" s="24" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="J7" s="24" t="s">
         <v>195</v>
       </c>
       <c r="K7" s="24" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="L7" s="24" t="s">
         <v>168</v>
@@ -2187,18 +2187,18 @@
       <c r="D8" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="E8" s="45"/>
+      <c r="E8" s="39"/>
       <c r="F8" s="24"/>
       <c r="G8" s="24"/>
       <c r="H8" s="24"/>
       <c r="I8" s="24" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="J8" s="24" t="s">
         <v>195</v>
       </c>
       <c r="K8" s="24" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="L8" s="24" t="s">
         <v>167</v>
@@ -2260,7 +2260,7 @@
       <c r="D9" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="E9" s="45" t="s">
+      <c r="E9" s="39" t="s">
         <v>211</v>
       </c>
       <c r="F9" s="36" t="s">
@@ -2271,13 +2271,13 @@
       </c>
       <c r="H9" s="24"/>
       <c r="I9" s="24" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="J9" s="24" t="s">
         <v>195</v>
       </c>
       <c r="K9" s="24" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="L9" s="24" t="s">
         <v>168</v>
@@ -2332,18 +2332,18 @@
       <c r="D10" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="E10" s="45"/>
+      <c r="E10" s="39"/>
       <c r="F10" s="24"/>
       <c r="G10" s="24"/>
       <c r="H10" s="24"/>
       <c r="I10" s="24" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="J10" s="24" t="s">
         <v>195</v>
       </c>
       <c r="K10" s="24" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="L10" s="24" t="s">
         <v>167</v>
@@ -2398,7 +2398,7 @@
       <c r="D11" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="E11" s="45" t="s">
+      <c r="E11" s="39" t="s">
         <v>211</v>
       </c>
       <c r="F11" s="36" t="s">
@@ -2409,13 +2409,13 @@
       </c>
       <c r="H11" s="24"/>
       <c r="I11" s="24" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="J11" s="24" t="s">
         <v>195</v>
       </c>
       <c r="K11" s="24" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="L11" s="24" t="s">
         <v>168</v>
@@ -2483,13 +2483,13 @@
         <v>205</v>
       </c>
       <c r="I12" s="24" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="J12" s="24" t="s">
         <v>195</v>
       </c>
       <c r="K12" s="24" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="L12" s="24" t="s">
         <v>167</v>
@@ -2548,13 +2548,13 @@
         <v>205</v>
       </c>
       <c r="I13" s="24" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="J13" s="24" t="s">
         <v>195</v>
       </c>
       <c r="K13" s="24" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="L13" s="24" t="s">
         <v>168</v>
@@ -2616,13 +2616,13 @@
         <v>213</v>
       </c>
       <c r="I14" s="24" t="s">
+        <v>209</v>
+      </c>
+      <c r="J14" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="J14" s="24" t="s">
+      <c r="K14" s="24" t="s">
         <v>215</v>
-      </c>
-      <c r="K14" s="24" t="s">
-        <v>209</v>
       </c>
       <c r="L14" s="24" t="s">
         <v>167</v>
@@ -2691,13 +2691,13 @@
         <v>213</v>
       </c>
       <c r="I15" s="24" t="s">
+        <v>209</v>
+      </c>
+      <c r="J15" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="J15" s="24" t="s">
+      <c r="K15" s="24" t="s">
         <v>215</v>
-      </c>
-      <c r="K15" s="24" t="s">
-        <v>209</v>
       </c>
       <c r="L15" s="24" t="s">
         <v>167</v>
@@ -14684,7 +14684,7 @@
           <x14:formula1>
             <xm:f>Dropdown!$H$2:$H$3</xm:f>
           </x14:formula1>
-          <xm:sqref>F16:G834 I16:L834 D16:D834</xm:sqref>
+          <xm:sqref>F16:G834 D16:D834 I16:K834 L16:L834</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{095226A7-BA7E-44B6-BA27-9F060F592E11}">
           <x14:formula1>
@@ -15509,13 +15509,13 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="71.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="43" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="43" t="s">
         <v>109</v>
       </c>
-      <c r="C2" s="42" t="s">
+      <c r="C2" s="43" t="s">
         <v>110</v>
       </c>
       <c r="D2" s="27" t="s">
@@ -15523,37 +15523,37 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="54.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="43"/>
-      <c r="B3" s="43"/>
-      <c r="C3" s="43"/>
+      <c r="A3" s="44"/>
+      <c r="B3" s="44"/>
+      <c r="C3" s="44"/>
       <c r="D3" s="27" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="78.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="43"/>
-      <c r="B4" s="43"/>
-      <c r="C4" s="43"/>
+      <c r="A4" s="44"/>
+      <c r="B4" s="44"/>
+      <c r="C4" s="44"/>
       <c r="D4" s="27" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="78.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="44"/>
-      <c r="B5" s="44"/>
-      <c r="C5" s="44"/>
+      <c r="A5" s="45"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="45"/>
       <c r="D5" s="27" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="39" t="s">
+      <c r="A6" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="39" t="s">
+      <c r="B6" s="40" t="s">
         <v>115</v>
       </c>
-      <c r="C6" s="39" t="s">
+      <c r="C6" s="40" t="s">
         <v>116</v>
       </c>
       <c r="D6" s="13" t="s">
@@ -15561,25 +15561,25 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="73.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="40"/>
-      <c r="B7" s="40"/>
-      <c r="C7" s="40"/>
+      <c r="A7" s="41"/>
+      <c r="B7" s="41"/>
+      <c r="C7" s="41"/>
       <c r="D7" s="13" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="73.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="40"/>
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
+      <c r="A8" s="41"/>
+      <c r="B8" s="41"/>
+      <c r="C8" s="41"/>
       <c r="D8" s="27" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="73.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="41"/>
-      <c r="B9" s="41"/>
-      <c r="C9" s="41"/>
+      <c r="A9" s="42"/>
+      <c r="B9" s="42"/>
+      <c r="C9" s="42"/>
       <c r="D9" s="27" t="s">
         <v>114</v>
       </c>
@@ -15676,13 +15676,13 @@
       </c>
     </row>
     <row r="17" spans="1:4" ht="77.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="39" t="s">
+      <c r="B17" s="40" t="s">
         <v>133</v>
       </c>
-      <c r="C17" s="39" t="s">
+      <c r="C17" s="40" t="s">
         <v>134</v>
       </c>
       <c r="D17" s="13" t="s">
@@ -15690,33 +15690,33 @@
       </c>
     </row>
     <row r="18" spans="1:4" ht="72.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="40"/>
-      <c r="B18" s="40"/>
-      <c r="C18" s="40"/>
+      <c r="A18" s="41"/>
+      <c r="B18" s="41"/>
+      <c r="C18" s="41"/>
       <c r="D18" s="13" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="78.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="40"/>
-      <c r="B19" s="40"/>
-      <c r="C19" s="40"/>
+      <c r="A19" s="41"/>
+      <c r="B19" s="41"/>
+      <c r="C19" s="41"/>
       <c r="D19" s="13" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="78.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="40"/>
-      <c r="B20" s="40"/>
-      <c r="C20" s="40"/>
+      <c r="A20" s="41"/>
+      <c r="B20" s="41"/>
+      <c r="C20" s="41"/>
       <c r="D20" s="13" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="78.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="41"/>
-      <c r="B21" s="41"/>
-      <c r="C21" s="41"/>
+      <c r="A21" s="42"/>
+      <c r="B21" s="42"/>
+      <c r="C21" s="42"/>
       <c r="D21" s="27" t="s">
         <v>114</v>
       </c>
@@ -15886,44 +15886,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Government_x0020_Body xmlns="b413c3fd-5a3b-4239-b985-69032e371c04" xsi:nil="true"/>
-    <Date_x0020_Opened xmlns="b413c3fd-5a3b-4239-b985-69032e371c04" xsi:nil="true"/>
-    <LegacyData xmlns="aaacb922-5235-4a66-b188-303b9b46fbd7" xsi:nil="true"/>
-    <Descriptor xmlns="0063f72e-ace3-48fb-9c1f-5b513408b31f" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ff8cd83-fc61-4182-af0d-9444b096b4cc"/>
-    <Invision xmlns="58eecf05-07e6-460c-a17a-1e6913e0d7ae">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Invision>
-    <m975189f4ba442ecbf67d4147307b177 xmlns="4ff8cd83-fc61-4182-af0d-9444b096b4cc">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </m975189f4ba442ecbf67d4147307b177>
-    <Security_x0020_Classification xmlns="0063f72e-ace3-48fb-9c1f-5b513408b31f" xsi:nil="true"/>
-    <ijmz xmlns="58eecf05-07e6-460c-a17a-1e6913e0d7ae" xsi:nil="true"/>
-    <Retention_x0020_Label xmlns="a8f60570-4bd3-4f2b-950b-a996de8ab151" xsi:nil="true"/>
-    <Date_x0020_Closed xmlns="b413c3fd-5a3b-4239-b985-69032e371c04" xsi:nil="true"/>
-    <_dlc_DocId xmlns="4ff8cd83-fc61-4182-af0d-9444b096b4cc" xsi:nil="true"/>
-    <_dlc_DocIdUrl xmlns="4ff8cd83-fc61-4182-af0d-9444b096b4cc">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </_dlc_DocIdUrl>
-    <Invisiondesigns xmlns="58eecf05-07e6-460c-a17a-1e6913e0d7ae" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
   <Receiver>
@@ -15971,6 +15933,44 @@
     <Filter/>
   </Receiver>
 </spe:Receivers>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Government_x0020_Body xmlns="b413c3fd-5a3b-4239-b985-69032e371c04" xsi:nil="true"/>
+    <Date_x0020_Opened xmlns="b413c3fd-5a3b-4239-b985-69032e371c04" xsi:nil="true"/>
+    <LegacyData xmlns="aaacb922-5235-4a66-b188-303b9b46fbd7" xsi:nil="true"/>
+    <Descriptor xmlns="0063f72e-ace3-48fb-9c1f-5b513408b31f" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ff8cd83-fc61-4182-af0d-9444b096b4cc"/>
+    <Invision xmlns="58eecf05-07e6-460c-a17a-1e6913e0d7ae">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Invision>
+    <m975189f4ba442ecbf67d4147307b177 xmlns="4ff8cd83-fc61-4182-af0d-9444b096b4cc">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </m975189f4ba442ecbf67d4147307b177>
+    <Security_x0020_Classification xmlns="0063f72e-ace3-48fb-9c1f-5b513408b31f" xsi:nil="true"/>
+    <ijmz xmlns="58eecf05-07e6-460c-a17a-1e6913e0d7ae" xsi:nil="true"/>
+    <Retention_x0020_Label xmlns="a8f60570-4bd3-4f2b-950b-a996de8ab151" xsi:nil="true"/>
+    <Date_x0020_Closed xmlns="b413c3fd-5a3b-4239-b985-69032e371c04" xsi:nil="true"/>
+    <_dlc_DocId xmlns="4ff8cd83-fc61-4182-af0d-9444b096b4cc" xsi:nil="true"/>
+    <_dlc_DocIdUrl xmlns="4ff8cd83-fc61-4182-af0d-9444b096b4cc">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </_dlc_DocIdUrl>
+    <Invisiondesigns xmlns="58eecf05-07e6-460c-a17a-1e6913e0d7ae" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
@@ -16342,6 +16342,22 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5AF44877-6D21-41C2-9736-04B57D725022}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6216EEDE-1870-4B1D-BF90-D3816A946FAF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBEDEBF5-0F8B-43D7-9E7F-E4CDAE2C086C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="b413c3fd-5a3b-4239-b985-69032e371c04"/>
@@ -16358,22 +16374,6 @@
     <ds:schemaRef ds:uri="0063f72e-ace3-48fb-9c1f-5b513408b31f"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6216EEDE-1870-4B1D-BF90-D3816A946FAF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5AF44877-6D21-41C2-9736-04B57D725022}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>